<commit_message>
rm useless line 2de46f743a40b54144598925b4c637c01abf16b0
</commit_message>
<xml_diff>
--- a/ig/update-practitioner-qualification/StructureDefinition-fr-core-practitioner.xlsx
+++ b/ig/update-practitioner-qualification/StructureDefinition-fr-core-practitioner.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2321" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2322" uniqueCount="490">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-06T14:52:13+00:00</t>
+    <t>2024-02-06T15:01:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -700,7 +700,10 @@
     <t>required</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/identifier-use</t>
+    <t>Identifies the purpose for this identifier, if known .</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/identifier-use|4.0.1</t>
   </si>
   <si>
     <t>Identifier.use</t>
@@ -4460,9 +4463,11 @@
       <c r="X23" t="s" s="2">
         <v>219</v>
       </c>
-      <c r="Y23" s="2"/>
+      <c r="Y23" t="s" s="2">
+        <v>220</v>
+      </c>
       <c r="Z23" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>77</v>
@@ -4480,7 +4485,7 @@
         <v>77</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
@@ -4498,7 +4503,7 @@
         <v>102</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AM23" t="s" s="2">
         <v>77</v>
@@ -4509,10 +4514,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4535,19 +4540,19 @@
         <v>89</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>77</v>
@@ -4576,7 +4581,7 @@
       </c>
       <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>77</v>
@@ -4594,7 +4599,7 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -4609,10 +4614,10 @@
         <v>101</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AM24" t="s" s="2">
         <v>77</v>
@@ -4623,10 +4628,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4735,10 +4740,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4849,10 +4854,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4878,16 +4883,16 @@
         <v>148</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="O27" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>77</v>
@@ -4936,7 +4941,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4951,10 +4956,10 @@
         <v>101</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>77</v>
@@ -4965,10 +4970,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5077,10 +5082,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5191,10 +5196,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5220,16 +5225,16 @@
         <v>132</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="O30" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>77</v>
@@ -5242,7 +5247,7 @@
         <v>77</v>
       </c>
       <c r="T30" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="U30" t="s" s="2">
         <v>77</v>
@@ -5278,7 +5283,7 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -5293,10 +5298,10 @@
         <v>101</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>77</v>
@@ -5307,10 +5312,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5336,13 +5341,13 @@
         <v>104</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
@@ -5392,7 +5397,7 @@
         <v>77</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -5407,10 +5412,10 @@
         <v>101</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>77</v>
@@ -5421,10 +5426,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5450,16 +5455,16 @@
         <v>172</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O32" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>77</v>
@@ -5508,7 +5513,7 @@
         <v>77</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -5523,10 +5528,10 @@
         <v>101</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>77</v>
@@ -5537,10 +5542,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5566,16 +5571,16 @@
         <v>104</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O33" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>77</v>
@@ -5624,7 +5629,7 @@
         <v>77</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5639,10 +5644,10 @@
         <v>101</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>77</v>
@@ -5653,10 +5658,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5679,19 +5684,19 @@
         <v>89</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>77</v>
@@ -5740,7 +5745,7 @@
         <v>77</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5755,10 +5760,10 @@
         <v>101</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AM34" t="s" s="2">
         <v>77</v>
@@ -5769,10 +5774,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5798,16 +5803,16 @@
         <v>104</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>77</v>
@@ -5856,7 +5861,7 @@
         <v>77</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5871,10 +5876,10 @@
         <v>101</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AM35" t="s" s="2">
         <v>77</v>
@@ -5885,10 +5890,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5914,16 +5919,16 @@
         <v>132</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>77</v>
@@ -5936,7 +5941,7 @@
         <v>77</v>
       </c>
       <c r="T36" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="U36" t="s" s="2">
         <v>77</v>
@@ -5972,7 +5977,7 @@
         <v>77</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5987,13 +5992,13 @@
         <v>101</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>77</v>
@@ -6001,10 +6006,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6030,13 +6035,13 @@
         <v>104</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -6050,7 +6055,7 @@
         <v>77</v>
       </c>
       <c r="T37" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="U37" t="s" s="2">
         <v>77</v>
@@ -6086,7 +6091,7 @@
         <v>77</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -6101,13 +6106,13 @@
         <v>101</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AN37" t="s" s="2">
         <v>77</v>
@@ -6115,10 +6120,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6141,16 +6146,16 @@
         <v>89</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6200,7 +6205,7 @@
         <v>77</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -6212,16 +6217,16 @@
         <v>100</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>77</v>
@@ -6229,10 +6234,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6255,16 +6260,16 @@
         <v>89</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
@@ -6314,7 +6319,7 @@
         <v>77</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -6326,16 +6331,16 @@
         <v>100</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AN39" t="s" s="2">
         <v>77</v>
@@ -6343,10 +6348,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6369,70 +6374,70 @@
         <v>89</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L40" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="M40" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="O40" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="P40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q40" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="R40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE40" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF40" t="s" s="2">
         <v>332</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>333</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="O40" t="s" s="2">
-        <v>335</v>
-      </c>
-      <c r="P40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q40" t="s" s="2">
-        <v>336</v>
-      </c>
-      <c r="R40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE40" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF40" t="s" s="2">
-        <v>331</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6450,21 +6455,21 @@
         <v>77</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AM40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6487,19 +6492,19 @@
         <v>77</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="O41" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="P41" t="s" s="2">
         <v>77</v>
@@ -6548,7 +6553,7 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6563,13 +6568,13 @@
         <v>101</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>77</v>
@@ -6577,10 +6582,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6603,19 +6608,19 @@
         <v>77</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="O42" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>77</v>
@@ -6664,7 +6669,7 @@
         <v>77</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6676,16 +6681,16 @@
         <v>100</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AN42" t="s" s="2">
         <v>77</v>
@@ -6693,10 +6698,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6805,10 +6810,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6919,13 +6924,13 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="B45" t="s" s="2">
         <v>360</v>
       </c>
-      <c r="B45" t="s" s="2">
-        <v>359</v>
-      </c>
       <c r="C45" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D45" t="s" s="2">
         <v>77</v>
@@ -6947,13 +6952,13 @@
         <v>77</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -7033,10 +7038,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7062,13 +7067,13 @@
         <v>172</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -7082,7 +7087,7 @@
         <v>77</v>
       </c>
       <c r="T46" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="U46" t="s" s="2">
         <v>77</v>
@@ -7097,10 +7102,10 @@
         <v>219</v>
       </c>
       <c r="Y46" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="Z46" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>77</v>
@@ -7118,7 +7123,7 @@
         <v>77</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -7127,19 +7132,19 @@
         <v>88</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>77</v>
@@ -7147,10 +7152,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7176,16 +7181,16 @@
         <v>104</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="O47" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="P47" t="s" s="2">
         <v>77</v>
@@ -7234,7 +7239,7 @@
         <v>77</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -7249,13 +7254,13 @@
         <v>101</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AN47" t="s" s="2">
         <v>77</v>
@@ -7263,10 +7268,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7292,16 +7297,16 @@
         <v>172</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="O48" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>77</v>
@@ -7329,10 +7334,10 @@
         <v>219</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>77</v>
@@ -7350,7 +7355,7 @@
         <v>77</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>78</v>
@@ -7365,13 +7370,13 @@
         <v>101</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="AN48" t="s" s="2">
         <v>77</v>
@@ -7379,10 +7384,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7405,16 +7410,16 @@
         <v>89</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="N49" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -7464,7 +7469,7 @@
         <v>77</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -7493,10 +7498,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7519,16 +7524,16 @@
         <v>89</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
@@ -7578,7 +7583,7 @@
         <v>77</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>78</v>
@@ -7590,16 +7595,16 @@
         <v>100</v>
       </c>
       <c r="AJ50" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="AK50" t="s" s="2">
         <v>102</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AM50" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="AN50" t="s" s="2">
         <v>77</v>
@@ -7607,10 +7612,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7633,19 +7638,19 @@
         <v>77</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="O51" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>77</v>
@@ -7694,7 +7699,7 @@
         <v>77</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>78</v>
@@ -7709,13 +7714,13 @@
         <v>101</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="AM51" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="AN51" t="s" s="2">
         <v>77</v>
@@ -7723,10 +7728,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7752,16 +7757,16 @@
         <v>172</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O52" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>77</v>
@@ -7790,7 +7795,7 @@
       </c>
       <c r="Y52" s="2"/>
       <c r="Z52" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>77</v>
@@ -7808,7 +7813,7 @@
         <v>77</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>78</v>
@@ -7823,13 +7828,13 @@
         <v>101</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="AL52" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="AN52" t="s" s="2">
         <v>77</v>
@@ -7837,10 +7842,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7863,17 +7868,17 @@
         <v>89</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>77</v>
@@ -7922,7 +7927,7 @@
         <v>77</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -7937,13 +7942,13 @@
         <v>101</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AN53" t="s" s="2">
         <v>77</v>
@@ -7951,10 +7956,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7977,19 +7982,19 @@
         <v>77</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="O54" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>77</v>
@@ -8038,7 +8043,7 @@
         <v>77</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
@@ -8050,16 +8055,16 @@
         <v>100</v>
       </c>
       <c r="AJ54" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="AN54" t="s" s="2">
         <v>77</v>
@@ -8067,10 +8072,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8093,13 +8098,13 @@
         <v>77</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8150,7 +8155,7 @@
         <v>77</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>78</v>
@@ -8165,13 +8170,13 @@
         <v>101</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AM55" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="AN55" t="s" s="2">
         <v>77</v>
@@ -8179,10 +8184,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8291,10 +8296,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8405,14 +8410,14 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
@@ -8434,10 +8439,10 @@
         <v>111</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="N58" t="s" s="2">
         <v>114</v>
@@ -8492,7 +8497,7 @@
         <v>77</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>78</v>
@@ -8521,10 +8526,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8550,14 +8555,14 @@
         <v>204</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>77</v>
@@ -8606,7 +8611,7 @@
         <v>77</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>78</v>
@@ -8621,13 +8626,13 @@
         <v>101</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="AL59" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="AM59" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="AN59" t="s" s="2">
         <v>77</v>
@@ -8635,10 +8640,10 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8661,16 +8666,16 @@
         <v>77</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -8700,7 +8705,7 @@
       </c>
       <c r="Y60" s="2"/>
       <c r="Z60" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="AA60" t="s" s="2">
         <v>77</v>
@@ -8718,7 +8723,7 @@
         <v>77</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>88</v>
@@ -8733,13 +8738,13 @@
         <v>101</v>
       </c>
       <c r="AK60" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="AL60" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AM60" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="AN60" t="s" s="2">
         <v>77</v>
@@ -8747,10 +8752,10 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8773,19 +8778,19 @@
         <v>77</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O61" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="P61" t="s" s="2">
         <v>77</v>
@@ -8834,7 +8839,7 @@
         <v>77</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>78</v>
@@ -8846,16 +8851,16 @@
         <v>100</v>
       </c>
       <c r="AJ61" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="AK61" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="AL61" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="AM61" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="AN61" t="s" s="2">
         <v>77</v>
@@ -8863,10 +8868,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8889,16 +8894,16 @@
         <v>77</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="N62" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
@@ -8948,7 +8953,7 @@
         <v>77</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>78</v>
@@ -8960,13 +8965,13 @@
         <v>100</v>
       </c>
       <c r="AJ62" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="AK62" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL62" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="AM62" t="s" s="2">
         <v>77</v>
@@ -8977,10 +8982,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9003,19 +9008,19 @@
         <v>77</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="N63" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="O63" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="P63" t="s" s="2">
         <v>77</v>
@@ -9064,7 +9069,7 @@
         <v>77</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>78</v>
@@ -9079,13 +9084,13 @@
         <v>101</v>
       </c>
       <c r="AK63" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="AM63" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="AN63" t="s" s="2">
         <v>77</v>

</xml_diff>

<commit_message>
rm useless lines 3bc79d0b9c4e3e921fce964afd729a862b5f2b77
</commit_message>
<xml_diff>
--- a/ig/update-practitioner-qualification/StructureDefinition-fr-core-practitioner.xlsx
+++ b/ig/update-practitioner-qualification/StructureDefinition-fr-core-practitioner.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2033" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2034" uniqueCount="443">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-06T15:40:57+00:00</t>
+    <t>2024-02-06T16:15:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1170,7 +1170,10 @@
     <t>Needed to address the person correctly.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/administrative-gender</t>
+    <t>The gender of a person used for administrative purposes.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/administrative-gender|4.0.1</t>
   </si>
   <si>
     <t>STF-5</t>
@@ -6732,9 +6735,11 @@
       <c r="X44" t="s" s="2">
         <v>219</v>
       </c>
-      <c r="Y44" s="2"/>
+      <c r="Y44" t="s" s="2">
+        <v>372</v>
+      </c>
       <c r="Z44" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>77</v>
@@ -6767,13 +6772,13 @@
         <v>101</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="AM44" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="AN44" t="s" s="2">
         <v>77</v>
@@ -6781,10 +6786,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6807,17 +6812,17 @@
         <v>89</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="P45" t="s" s="2">
         <v>77</v>
@@ -6866,7 +6871,7 @@
         <v>77</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -6881,13 +6886,13 @@
         <v>101</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>77</v>
@@ -6895,10 +6900,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6921,19 +6926,19 @@
         <v>77</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="O46" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="P46" t="s" s="2">
         <v>77</v>
@@ -6982,7 +6987,7 @@
         <v>77</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -6994,16 +6999,16 @@
         <v>100</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>77</v>
@@ -7011,10 +7016,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7037,13 +7042,13 @@
         <v>77</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7094,7 +7099,7 @@
         <v>77</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -7109,13 +7114,13 @@
         <v>101</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="AN47" t="s" s="2">
         <v>77</v>
@@ -7123,10 +7128,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7235,10 +7240,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7349,14 +7354,14 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
@@ -7378,10 +7383,10 @@
         <v>111</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="N50" t="s" s="2">
         <v>114</v>
@@ -7436,7 +7441,7 @@
         <v>77</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>78</v>
@@ -7465,10 +7470,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7494,14 +7499,14 @@
         <v>204</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>77</v>
@@ -7550,7 +7555,7 @@
         <v>77</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>78</v>
@@ -7565,13 +7570,13 @@
         <v>101</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="AM51" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="AN51" t="s" s="2">
         <v>77</v>
@@ -7579,10 +7584,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7608,13 +7613,13 @@
         <v>225</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -7644,7 +7649,7 @@
       </c>
       <c r="Y52" s="2"/>
       <c r="Z52" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>77</v>
@@ -7662,7 +7667,7 @@
         <v>77</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>88</v>
@@ -7677,13 +7682,13 @@
         <v>101</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="AL52" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="AN52" t="s" s="2">
         <v>77</v>
@@ -7691,10 +7696,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7720,16 +7725,16 @@
         <v>313</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="N53" t="s" s="2">
         <v>316</v>
       </c>
       <c r="O53" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>77</v>
@@ -7778,7 +7783,7 @@
         <v>77</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -7793,13 +7798,13 @@
         <v>318</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="AN53" t="s" s="2">
         <v>77</v>
@@ -7807,10 +7812,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7836,13 +7841,13 @@
         <v>323</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
@@ -7892,7 +7897,7 @@
         <v>77</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
@@ -7910,7 +7915,7 @@
         <v>77</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="AM54" t="s" s="2">
         <v>77</v>
@@ -7921,10 +7926,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -7950,16 +7955,16 @@
         <v>225</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="O55" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>77</v>
@@ -8008,7 +8013,7 @@
         <v>77</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>78</v>
@@ -8023,13 +8028,13 @@
         <v>101</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="AM55" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="AN55" t="s" s="2">
         <v>77</v>

</xml_diff>

<commit_message>
add qualification short example d05eb4db29caf791e9cfa1d4f30f8e2c2a36321f
</commit_message>
<xml_diff>
--- a/ig/update-practitioner-qualification/StructureDefinition-fr-core-practitioner.xlsx
+++ b/ig/update-practitioner-qualification/StructureDefinition-fr-core-practitioner.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-06T16:15:17+00:00</t>
+    <t>2024-02-12T12:39:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1249,10 +1249,10 @@
 </t>
   </si>
   <si>
-    <t>Qualifications obtained by training and certification/Diplômes</t>
-  </si>
-  <si>
-    <t>Qualifications obtained by training and certification/Diplômes obtenus</t>
+    <t>Qualifications obtained by training and certification | Diplômes. Les différents diplômes sont : les diplômes d'état français, les commissions de qualification, les diplômes d'études spécialisées, les DESC groupe 1 et 2, les capacités, les diplômes d'un pays de l'EEE, les diplômes d'université (DU) ou Inter-Universitaire, les certificats d'étude spéciale, les attestations, les diplômes européens d'études spécialisées, les diplômes de 2ème cycle non qualifiant et les autres types de diplômes. Pour plus d'informations, consulter le jeu de valeurs associé.</t>
+  </si>
+  <si>
+    <t>The official certifications, training, and licenses that authorize or otherwise pertain to the provision of care by the practitioner.  For example, a medical license issued by a medical board authorizing the practitioner to practice medicine within a certian locality.</t>
   </si>
   <si>
     <t>CER?</t>

</xml_diff>